<commit_message>
titles and devices name  fixes
</commit_message>
<xml_diff>
--- a/api/placeholders/RifResistanceRate.xlsx
+++ b/api/placeholders/RifResistanceRate.xlsx
@@ -26,9 +26,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
-    <t>Deployment Name</t>
-  </si>
-  <si>
     <t>Total Tests</t>
   </si>
   <si>
@@ -117,6 +114,9 @@
   </si>
   <si>
     <t>Wooster Hospital</t>
+  </si>
+  <si>
+    <t>Devices</t>
   </si>
 </sst>
 </file>
@@ -772,14 +772,14 @@
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
@@ -790,36 +790,36 @@
     </row>
     <row r="7" spans="1:7" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="38" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>1</v>
-      </c>
       <c r="E7" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="G7" s="38" t="s">
         <v>4</v>
-      </c>
-      <c r="G7" s="38" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="D8" s="6">
         <v>1927</v>
@@ -836,13 +836,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="D9" s="9">
         <v>45</v>
@@ -859,13 +859,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="33" t="s">
         <v>15</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>16</v>
       </c>
       <c r="D10" s="12">
         <v>1011</v>
@@ -882,13 +882,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="C11" s="33" t="s">
         <v>18</v>
-      </c>
-      <c r="C11" s="33" t="s">
-        <v>19</v>
       </c>
       <c r="D11" s="15">
         <v>24</v>
@@ -905,13 +905,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="33" t="s">
         <v>20</v>
-      </c>
-      <c r="B12" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>21</v>
       </c>
       <c r="D12" s="18">
         <v>2130</v>
@@ -928,13 +928,13 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="33" t="s">
         <v>10</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>11</v>
       </c>
       <c r="D13" s="21">
         <v>2063</v>
@@ -951,13 +951,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="33" t="s">
         <v>23</v>
-      </c>
-      <c r="B14" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="33" t="s">
-        <v>24</v>
       </c>
       <c r="D14" s="24">
         <v>2653</v>
@@ -974,13 +974,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="C15" s="33" t="s">
         <v>26</v>
-      </c>
-      <c r="C15" s="33" t="s">
-        <v>27</v>
       </c>
       <c r="D15" s="27">
         <v>5</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="33" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="33" t="s">
-        <v>29</v>
       </c>
       <c r="D16" s="30">
         <v>4</v>
@@ -1020,13 +1020,13 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D17" s="34">
         <v>44</v>

</xml_diff>